<commit_message>
Análisis de nubes de palabras, correlación de longitud, BERTopic preliminar y dependencias
</commit_message>
<xml_diff>
--- a/data/utilities/stopwords.xlsx
+++ b/data/utilities/stopwords.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP ENVY\Documents\Maestria_MINE\SEMESTRE 4\3.OpcionGrado--Wilmer\capstonenlpencuestas_mine9\data\raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Acer\OneDrive\Escritorio\MINE009_Externado\CAPSTONE_U_EXTERNADO\capstonenlpencuestas_mine9\data\utilities\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{138F49CD-6133-48DC-9526-DAC5293B4E39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="21840" windowHeight="13290" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="21840" windowHeight="13290"/>
   </bookViews>
   <sheets>
     <sheet name="globales" sheetId="2" r:id="rId1"/>
@@ -26,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="61">
   <si>
     <t>encuesta</t>
   </si>
@@ -206,12 +205,15 @@
   </si>
   <si>
     <t>por favor</t>
+  </si>
+  <si>
+    <t>mas</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -522,15 +524,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{789E5CAB-B981-4237-B9FF-37E40AC0E671}">
-  <dimension ref="A1:B27"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B28"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.453125" customWidth="1"/>
-    <col min="2" max="2" width="22.6328125" customWidth="1"/>
+    <col min="1" max="1" width="26.42578125" customWidth="1"/>
+    <col min="2" max="2" width="22.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -538,7 +540,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>33</v>
       </c>
@@ -546,7 +548,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>33</v>
       </c>
@@ -554,7 +556,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>33</v>
       </c>
@@ -562,7 +564,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>33</v>
       </c>
@@ -570,7 +572,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>33</v>
       </c>
@@ -578,7 +580,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>33</v>
       </c>
@@ -586,7 +588,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>33</v>
       </c>
@@ -594,7 +596,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>33</v>
       </c>
@@ -602,7 +604,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>33</v>
       </c>
@@ -610,7 +612,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>33</v>
       </c>
@@ -618,7 +620,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>33</v>
       </c>
@@ -626,7 +628,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>33</v>
       </c>
@@ -634,7 +636,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>33</v>
       </c>
@@ -642,7 +644,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>33</v>
       </c>
@@ -650,7 +652,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>33</v>
       </c>
@@ -658,7 +660,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>33</v>
       </c>
@@ -666,7 +668,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>33</v>
       </c>
@@ -674,7 +676,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>33</v>
       </c>
@@ -682,7 +684,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>33</v>
       </c>
@@ -690,7 +692,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>33</v>
       </c>
@@ -698,7 +700,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>33</v>
       </c>
@@ -706,7 +708,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>33</v>
       </c>
@@ -714,7 +716,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>33</v>
       </c>
@@ -722,7 +724,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>33</v>
       </c>
@@ -730,7 +732,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>33</v>
       </c>
@@ -738,12 +740,20 @@
         <v>58</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>33</v>
       </c>
       <c r="B27" t="s">
         <v>59</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>33</v>
+      </c>
+      <c r="B28" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -753,15 +763,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B76"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.36328125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.26953125" customWidth="1"/>
+    <col min="1" max="1" width="30.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -769,7 +779,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -777,7 +787,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -785,7 +795,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -793,7 +803,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -801,7 +811,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -809,7 +819,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>2</v>
       </c>
@@ -817,7 +827,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>2</v>
       </c>
@@ -825,7 +835,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>2</v>
       </c>
@@ -833,7 +843,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -841,7 +851,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>2</v>
       </c>
@@ -849,7 +859,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>2</v>
       </c>
@@ -857,7 +867,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>2</v>
       </c>
@@ -865,7 +875,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>2</v>
       </c>
@@ -873,7 +883,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>2</v>
       </c>
@@ -881,7 +891,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>2</v>
       </c>
@@ -889,7 +899,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>2</v>
       </c>
@@ -897,7 +907,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>2</v>
       </c>
@@ -905,7 +915,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>20</v>
       </c>
@@ -913,7 +923,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>20</v>
       </c>
@@ -921,7 +931,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -929,7 +939,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>20</v>
       </c>
@@ -937,7 +947,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>20</v>
       </c>
@@ -945,7 +955,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>20</v>
       </c>
@@ -953,7 +963,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>20</v>
       </c>
@@ -961,7 +971,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>20</v>
       </c>
@@ -969,7 +979,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>20</v>
       </c>
@@ -977,7 +987,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>26</v>
       </c>
@@ -985,7 +995,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>26</v>
       </c>
@@ -993,7 +1003,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>26</v>
       </c>
@@ -1001,7 +1011,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>26</v>
       </c>
@@ -1009,7 +1019,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>26</v>
       </c>
@@ -1017,7 +1027,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>26</v>
       </c>
@@ -1025,7 +1035,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>26</v>
       </c>
@@ -1033,7 +1043,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>26</v>
       </c>
@@ -1041,7 +1051,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>26</v>
       </c>
@@ -1049,7 +1059,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>28</v>
       </c>
@@ -1057,7 +1067,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>28</v>
       </c>
@@ -1065,7 +1075,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>28</v>
       </c>
@@ -1073,7 +1083,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>28</v>
       </c>
@@ -1081,7 +1091,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>28</v>
       </c>
@@ -1089,7 +1099,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>28</v>
       </c>
@@ -1097,7 +1107,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>28</v>
       </c>
@@ -1105,7 +1115,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>28</v>
       </c>
@@ -1113,7 +1123,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>28</v>
       </c>
@@ -1121,7 +1131,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>28</v>
       </c>
@@ -1129,7 +1139,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>30</v>
       </c>
@@ -1137,7 +1147,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>30</v>
       </c>
@@ -1145,7 +1155,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>30</v>
       </c>
@@ -1153,7 +1163,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>30</v>
       </c>
@@ -1161,7 +1171,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>30</v>
       </c>
@@ -1169,7 +1179,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>30</v>
       </c>
@@ -1177,7 +1187,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>30</v>
       </c>
@@ -1185,7 +1195,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>30</v>
       </c>
@@ -1193,7 +1203,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>30</v>
       </c>
@@ -1201,7 +1211,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>30</v>
       </c>
@@ -1209,7 +1219,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>31</v>
       </c>
@@ -1217,7 +1227,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>31</v>
       </c>
@@ -1225,7 +1235,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>31</v>
       </c>
@@ -1233,7 +1243,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>31</v>
       </c>
@@ -1241,7 +1251,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>31</v>
       </c>
@@ -1249,7 +1259,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>31</v>
       </c>
@@ -1257,7 +1267,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>31</v>
       </c>
@@ -1265,7 +1275,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>31</v>
       </c>
@@ -1273,7 +1283,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>31</v>
       </c>
@@ -1281,7 +1291,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>31</v>
       </c>
@@ -1289,7 +1299,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>32</v>
       </c>
@@ -1297,7 +1307,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>32</v>
       </c>
@@ -1305,7 +1315,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>32</v>
       </c>
@@ -1313,7 +1323,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>32</v>
       </c>
@@ -1321,7 +1331,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>32</v>
       </c>
@@ -1329,7 +1339,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>32</v>
       </c>
@@ -1337,7 +1347,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>32</v>
       </c>
@@ -1345,7 +1355,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>32</v>
       </c>
@@ -1353,7 +1363,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>32</v>
       </c>
@@ -1361,7 +1371,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>32</v>
       </c>

</xml_diff>

<commit_message>
conservacion adverbios para analisis sentimientos
</commit_message>
<xml_diff>
--- a/data/utilities/stopwords.xlsx
+++ b/data/utilities/stopwords.xlsx
@@ -1,19 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Acer\OneDrive\Escritorio\MINE009_Externado\CAPSTONE_U_EXTERNADO\capstonenlpencuestas_mine9\data\utilities\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP ENVY\Documents\Maestria_MINE\SEMESTRE 4\3.OpcionGrado--Wilmer\capstonenlpencuestas_mine9\data\utilities\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{676BE8B3-CDF8-48AF-908D-1758725BA35E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="21840" windowHeight="13290"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="21840" windowHeight="13290" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="globales" sheetId="2" r:id="rId1"/>
     <sheet name="particulares" sheetId="1" r:id="rId2"/>
+    <sheet name="adverbios" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="127">
   <si>
     <t>encuesta</t>
   </si>
@@ -208,12 +210,210 @@
   </si>
   <si>
     <t>mas</t>
+  </si>
+  <si>
+    <t>adverbios</t>
+  </si>
+  <si>
+    <t>abajo</t>
+  </si>
+  <si>
+    <t>acaso</t>
+  </si>
+  <si>
+    <t>afuera</t>
+  </si>
+  <si>
+    <t>ahi</t>
+  </si>
+  <si>
+    <t>ahora</t>
+  </si>
+  <si>
+    <t>alli</t>
+  </si>
+  <si>
+    <t>alrededor</t>
+  </si>
+  <si>
+    <t>anoche</t>
+  </si>
+  <si>
+    <t>antes</t>
+  </si>
+  <si>
+    <t>aqui</t>
+  </si>
+  <si>
+    <t>arriba</t>
+  </si>
+  <si>
+    <t>asi</t>
+  </si>
+  <si>
+    <t>bastante</t>
+  </si>
+  <si>
+    <t>bien</t>
+  </si>
+  <si>
+    <t>casi</t>
+  </si>
+  <si>
+    <t>cerca</t>
+  </si>
+  <si>
+    <t>ciertamente</t>
+  </si>
+  <si>
+    <t>claramente</t>
+  </si>
+  <si>
+    <t>cuando</t>
+  </si>
+  <si>
+    <t>demasiado</t>
+  </si>
+  <si>
+    <t>dentro</t>
+  </si>
+  <si>
+    <t>delante</t>
+  </si>
+  <si>
+    <t>deprisa</t>
+  </si>
+  <si>
+    <t>desde</t>
+  </si>
+  <si>
+    <t>despacio</t>
+  </si>
+  <si>
+    <t>despues</t>
+  </si>
+  <si>
+    <t>detras</t>
+  </si>
+  <si>
+    <t>donde</t>
+  </si>
+  <si>
+    <t>efectivamente</t>
+  </si>
+  <si>
+    <t>enfrente</t>
+  </si>
+  <si>
+    <t>exactamente</t>
+  </si>
+  <si>
+    <t>facilmente</t>
+  </si>
+  <si>
+    <t>fuera</t>
+  </si>
+  <si>
+    <t>hoy</t>
+  </si>
+  <si>
+    <t>jamas</t>
+  </si>
+  <si>
+    <t>lentamente</t>
+  </si>
+  <si>
+    <t>lejos</t>
+  </si>
+  <si>
+    <t>mal</t>
+  </si>
+  <si>
+    <t>manana</t>
+  </si>
+  <si>
+    <t>mayormente</t>
+  </si>
+  <si>
+    <t>mejor</t>
+  </si>
+  <si>
+    <t>menos</t>
+  </si>
+  <si>
+    <t>mucho</t>
+  </si>
+  <si>
+    <t>naturalmente</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>nunca</t>
+  </si>
+  <si>
+    <t>obvio</t>
+  </si>
+  <si>
+    <t>peor</t>
+  </si>
+  <si>
+    <t>poco</t>
+  </si>
+  <si>
+    <t>probablemente</t>
+  </si>
+  <si>
+    <t>pronto</t>
+  </si>
+  <si>
+    <t>quizas</t>
+  </si>
+  <si>
+    <t>rapidamente</t>
+  </si>
+  <si>
+    <t>si</t>
+  </si>
+  <si>
+    <t>siempre</t>
+  </si>
+  <si>
+    <t>tal vez</t>
+  </si>
+  <si>
+    <t>tampoco</t>
+  </si>
+  <si>
+    <t>tarde</t>
+  </si>
+  <si>
+    <t>tanto</t>
+  </si>
+  <si>
+    <t>temprano</t>
+  </si>
+  <si>
+    <t>todavia</t>
+  </si>
+  <si>
+    <t>ultimamente</t>
+  </si>
+  <si>
+    <t>unicamente</t>
+  </si>
+  <si>
+    <t>verdaderamente</t>
+  </si>
+  <si>
+    <t>ya</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -249,7 +449,18 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -524,15 +735,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B28"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B24"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" customWidth="1"/>
-    <col min="2" max="2" width="22.5703125" customWidth="1"/>
+    <col min="1" max="1" width="26.453125" customWidth="1"/>
+    <col min="2" max="2" width="22.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -540,7 +751,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>33</v>
       </c>
@@ -548,7 +759,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>33</v>
       </c>
@@ -556,7 +767,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>33</v>
       </c>
@@ -564,7 +775,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>33</v>
       </c>
@@ -572,7 +783,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>33</v>
       </c>
@@ -580,180 +791,148 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>33</v>
       </c>
       <c r="B7" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>33</v>
       </c>
       <c r="B8" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>33</v>
       </c>
       <c r="B9" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>33</v>
       </c>
       <c r="B10" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>33</v>
       </c>
       <c r="B11" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>33</v>
       </c>
       <c r="B12" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>33</v>
       </c>
       <c r="B13" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>33</v>
       </c>
       <c r="B14" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>33</v>
       </c>
       <c r="B15" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>33</v>
       </c>
       <c r="B16" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>33</v>
       </c>
       <c r="B17" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>33</v>
       </c>
       <c r="B18" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>33</v>
       </c>
       <c r="B19" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>33</v>
       </c>
       <c r="B20" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>33</v>
       </c>
       <c r="B21" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>33</v>
       </c>
       <c r="B22" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>33</v>
       </c>
       <c r="B23" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>33</v>
       </c>
       <c r="B24" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>33</v>
-      </c>
-      <c r="B25" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>33</v>
-      </c>
-      <c r="B26" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>33</v>
-      </c>
-      <c r="B27" t="s">
         <v>59</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>33</v>
-      </c>
-      <c r="B28" t="s">
-        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -763,15 +942,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B76"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="30.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.28515625" customWidth="1"/>
+    <col min="1" max="1" width="30.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -779,7 +958,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -787,7 +966,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -795,7 +974,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -803,7 +982,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -811,7 +990,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -819,7 +998,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>2</v>
       </c>
@@ -827,7 +1006,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>2</v>
       </c>
@@ -835,7 +1014,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>2</v>
       </c>
@@ -843,7 +1022,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -851,7 +1030,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>2</v>
       </c>
@@ -859,7 +1038,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>2</v>
       </c>
@@ -867,7 +1046,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>2</v>
       </c>
@@ -875,7 +1054,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>2</v>
       </c>
@@ -883,7 +1062,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>2</v>
       </c>
@@ -891,7 +1070,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>2</v>
       </c>
@@ -899,7 +1078,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>2</v>
       </c>
@@ -907,7 +1086,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>2</v>
       </c>
@@ -915,7 +1094,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>20</v>
       </c>
@@ -923,7 +1102,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>20</v>
       </c>
@@ -931,7 +1110,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -939,7 +1118,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>20</v>
       </c>
@@ -947,7 +1126,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>20</v>
       </c>
@@ -955,7 +1134,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>20</v>
       </c>
@@ -963,7 +1142,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>20</v>
       </c>
@@ -971,7 +1150,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>20</v>
       </c>
@@ -979,7 +1158,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>20</v>
       </c>
@@ -987,7 +1166,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>26</v>
       </c>
@@ -995,7 +1174,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>26</v>
       </c>
@@ -1003,7 +1182,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>26</v>
       </c>
@@ -1011,7 +1190,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>26</v>
       </c>
@@ -1019,7 +1198,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>26</v>
       </c>
@@ -1027,7 +1206,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>26</v>
       </c>
@@ -1035,7 +1214,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>26</v>
       </c>
@@ -1043,7 +1222,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>26</v>
       </c>
@@ -1051,7 +1230,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>26</v>
       </c>
@@ -1059,7 +1238,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>28</v>
       </c>
@@ -1067,7 +1246,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>28</v>
       </c>
@@ -1075,7 +1254,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>28</v>
       </c>
@@ -1083,7 +1262,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>28</v>
       </c>
@@ -1091,7 +1270,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>28</v>
       </c>
@@ -1099,7 +1278,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>28</v>
       </c>
@@ -1107,7 +1286,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>28</v>
       </c>
@@ -1115,7 +1294,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>28</v>
       </c>
@@ -1123,7 +1302,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>28</v>
       </c>
@@ -1131,7 +1310,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>28</v>
       </c>
@@ -1139,7 +1318,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>30</v>
       </c>
@@ -1147,7 +1326,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>30</v>
       </c>
@@ -1155,7 +1334,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>30</v>
       </c>
@@ -1163,7 +1342,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>30</v>
       </c>
@@ -1171,7 +1350,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>30</v>
       </c>
@@ -1179,7 +1358,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>30</v>
       </c>
@@ -1187,7 +1366,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>30</v>
       </c>
@@ -1195,7 +1374,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>30</v>
       </c>
@@ -1203,7 +1382,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>30</v>
       </c>
@@ -1211,7 +1390,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>30</v>
       </c>
@@ -1219,7 +1398,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>31</v>
       </c>
@@ -1227,7 +1406,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>31</v>
       </c>
@@ -1235,7 +1414,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>31</v>
       </c>
@@ -1243,7 +1422,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>31</v>
       </c>
@@ -1251,7 +1430,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>31</v>
       </c>
@@ -1259,7 +1438,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>31</v>
       </c>
@@ -1267,7 +1446,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>31</v>
       </c>
@@ -1275,7 +1454,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>31</v>
       </c>
@@ -1283,7 +1462,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>31</v>
       </c>
@@ -1291,7 +1470,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>31</v>
       </c>
@@ -1299,7 +1478,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>32</v>
       </c>
@@ -1307,7 +1486,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>32</v>
       </c>
@@ -1315,7 +1494,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>32</v>
       </c>
@@ -1323,7 +1502,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>32</v>
       </c>
@@ -1331,7 +1510,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>32</v>
       </c>
@@ -1339,7 +1518,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>32</v>
       </c>
@@ -1347,7 +1526,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>32</v>
       </c>
@@ -1355,7 +1534,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>32</v>
       </c>
@@ -1363,7 +1542,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>32</v>
       </c>
@@ -1371,12 +1550,590 @@
         <v>29</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>32</v>
       </c>
       <c r="B76" t="s">
         <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B07C7C0B-433F-45E0-943A-A43C33B854D3}">
+  <dimension ref="A1:B71"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>61</v>
+      </c>
+      <c r="B6" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>61</v>
+      </c>
+      <c r="B7" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B8" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>61</v>
+      </c>
+      <c r="B9" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B12" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>61</v>
+      </c>
+      <c r="B13" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>61</v>
+      </c>
+      <c r="B14" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>61</v>
+      </c>
+      <c r="B15" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>61</v>
+      </c>
+      <c r="B16" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>61</v>
+      </c>
+      <c r="B17" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>61</v>
+      </c>
+      <c r="B18" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>61</v>
+      </c>
+      <c r="B19" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>61</v>
+      </c>
+      <c r="B20" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>61</v>
+      </c>
+      <c r="B21" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>61</v>
+      </c>
+      <c r="B22" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>61</v>
+      </c>
+      <c r="B23" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>61</v>
+      </c>
+      <c r="B24" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>61</v>
+      </c>
+      <c r="B25" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>61</v>
+      </c>
+      <c r="B26" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>61</v>
+      </c>
+      <c r="B27" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>61</v>
+      </c>
+      <c r="B28" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>61</v>
+      </c>
+      <c r="B29" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>61</v>
+      </c>
+      <c r="B30" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>61</v>
+      </c>
+      <c r="B31" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>61</v>
+      </c>
+      <c r="B32" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>61</v>
+      </c>
+      <c r="B33" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>61</v>
+      </c>
+      <c r="B34" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>61</v>
+      </c>
+      <c r="B35" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>61</v>
+      </c>
+      <c r="B36" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>61</v>
+      </c>
+      <c r="B37" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>61</v>
+      </c>
+      <c r="B38" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>61</v>
+      </c>
+      <c r="B39" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>61</v>
+      </c>
+      <c r="B40" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>61</v>
+      </c>
+      <c r="B41" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>61</v>
+      </c>
+      <c r="B42" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>61</v>
+      </c>
+      <c r="B43" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>61</v>
+      </c>
+      <c r="B44" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>61</v>
+      </c>
+      <c r="B45" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>61</v>
+      </c>
+      <c r="B46" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>61</v>
+      </c>
+      <c r="B47" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>61</v>
+      </c>
+      <c r="B48" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>61</v>
+      </c>
+      <c r="B49" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>61</v>
+      </c>
+      <c r="B50" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>61</v>
+      </c>
+      <c r="B51" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
+        <v>61</v>
+      </c>
+      <c r="B52" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>61</v>
+      </c>
+      <c r="B53" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>61</v>
+      </c>
+      <c r="B54" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
+        <v>61</v>
+      </c>
+      <c r="B55" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
+        <v>61</v>
+      </c>
+      <c r="B56" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
+        <v>61</v>
+      </c>
+      <c r="B57" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
+        <v>61</v>
+      </c>
+      <c r="B58" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
+        <v>61</v>
+      </c>
+      <c r="B59" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
+        <v>61</v>
+      </c>
+      <c r="B60" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
+        <v>61</v>
+      </c>
+      <c r="B61" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
+        <v>61</v>
+      </c>
+      <c r="B62" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
+        <v>61</v>
+      </c>
+      <c r="B63" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
+        <v>61</v>
+      </c>
+      <c r="B64" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
+        <v>61</v>
+      </c>
+      <c r="B65" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
+        <v>61</v>
+      </c>
+      <c r="B66" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
+        <v>61</v>
+      </c>
+      <c r="B67" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
+        <v>61</v>
+      </c>
+      <c r="B68" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
+        <v>61</v>
+      </c>
+      <c r="B69" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
+        <v>61</v>
+      </c>
+      <c r="B70" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
+        <v>61</v>
+      </c>
+      <c r="B71" t="s">
+        <v>126</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
debug 2 en pruebas_explorar_2.ipynb
</commit_message>
<xml_diff>
--- a/data/utilities/stopwords.xlsx
+++ b/data/utilities/stopwords.xlsx
@@ -8,15 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP ENVY\Documents\Maestria_MINE\SEMESTRE 4\3.OpcionGrado--Wilmer\capstonenlpencuestas_mine9\data\utilities\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{676BE8B3-CDF8-48AF-908D-1758725BA35E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEDDEC1E-A5C8-4DC5-904C-0D37DC84C3F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="21840" windowHeight="13290" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="globales" sheetId="2" r:id="rId1"/>
     <sheet name="particulares" sheetId="1" r:id="rId2"/>
     <sheet name="adverbios" sheetId="3" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">globales!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">particulares!$A$1:$B$1</definedName>
+  </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -27,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="149">
   <si>
     <t>encuesta</t>
   </si>
@@ -408,6 +412,72 @@
   </si>
   <si>
     <t>ya</t>
+  </si>
+  <si>
+    <t>maestro</t>
+  </si>
+  <si>
+    <t>maestra</t>
+  </si>
+  <si>
+    <t>maestros</t>
+  </si>
+  <si>
+    <t>maestras</t>
+  </si>
+  <si>
+    <t>doctor</t>
+  </si>
+  <si>
+    <t>doctora</t>
+  </si>
+  <si>
+    <t>doctores</t>
+  </si>
+  <si>
+    <t>catedratica</t>
+  </si>
+  <si>
+    <t>catedratico</t>
+  </si>
+  <si>
+    <t>pedagogo</t>
+  </si>
+  <si>
+    <t>pedagoga</t>
+  </si>
+  <si>
+    <t>educador</t>
+  </si>
+  <si>
+    <t>educadora</t>
+  </si>
+  <si>
+    <t>educadores</t>
+  </si>
+  <si>
+    <t>alumna</t>
+  </si>
+  <si>
+    <t>alumno</t>
+  </si>
+  <si>
+    <t>alumnos</t>
+  </si>
+  <si>
+    <t>alumnas</t>
+  </si>
+  <si>
+    <t>discipulo</t>
+  </si>
+  <si>
+    <t>discipula</t>
+  </si>
+  <si>
+    <t>aprendizaje</t>
+  </si>
+  <si>
+    <t>na</t>
   </si>
 </sst>
 </file>
@@ -449,18 +519,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -736,7 +795,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="26.453125" customWidth="1"/>
@@ -756,7 +815,7 @@
         <v>33</v>
       </c>
       <c r="B2" t="s">
-        <v>34</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
@@ -764,7 +823,7 @@
         <v>33</v>
       </c>
       <c r="B3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -772,7 +831,7 @@
         <v>33</v>
       </c>
       <c r="B4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
@@ -780,7 +839,7 @@
         <v>33</v>
       </c>
       <c r="B5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
@@ -788,7 +847,7 @@
         <v>33</v>
       </c>
       <c r="B6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
@@ -796,7 +855,7 @@
         <v>33</v>
       </c>
       <c r="B7" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
@@ -804,7 +863,7 @@
         <v>33</v>
       </c>
       <c r="B8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
@@ -812,7 +871,7 @@
         <v>33</v>
       </c>
       <c r="B9" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
@@ -820,7 +879,7 @@
         <v>33</v>
       </c>
       <c r="B10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
@@ -828,7 +887,7 @@
         <v>33</v>
       </c>
       <c r="B11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
@@ -836,7 +895,7 @@
         <v>33</v>
       </c>
       <c r="B12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
@@ -844,7 +903,7 @@
         <v>33</v>
       </c>
       <c r="B13" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
@@ -852,7 +911,7 @@
         <v>33</v>
       </c>
       <c r="B14" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
@@ -860,7 +919,7 @@
         <v>33</v>
       </c>
       <c r="B15" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
@@ -868,7 +927,7 @@
         <v>33</v>
       </c>
       <c r="B16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
@@ -876,7 +935,7 @@
         <v>33</v>
       </c>
       <c r="B17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
@@ -884,7 +943,7 @@
         <v>33</v>
       </c>
       <c r="B18" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
@@ -892,7 +951,7 @@
         <v>33</v>
       </c>
       <c r="B19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
@@ -900,7 +959,7 @@
         <v>33</v>
       </c>
       <c r="B20" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
@@ -908,7 +967,7 @@
         <v>33</v>
       </c>
       <c r="B21" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
@@ -916,7 +975,7 @@
         <v>33</v>
       </c>
       <c r="B22" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.35">
@@ -924,7 +983,7 @@
         <v>33</v>
       </c>
       <c r="B23" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.35">
@@ -932,10 +991,19 @@
         <v>33</v>
       </c>
       <c r="B24" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>33</v>
+      </c>
+      <c r="B25" t="s">
         <v>59</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:B1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -943,7 +1011,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B76"/>
+  <dimension ref="A1:B97"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30.453125" bestFit="1" customWidth="1"/>
@@ -971,7 +1039,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>4</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
@@ -979,7 +1047,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>5</v>
+        <v>139</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
@@ -987,7 +1055,7 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
+        <v>140</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
@@ -995,7 +1063,7 @@
         <v>2</v>
       </c>
       <c r="B6" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
@@ -1003,7 +1071,7 @@
         <v>2</v>
       </c>
       <c r="B7" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
@@ -1011,7 +1079,7 @@
         <v>2</v>
       </c>
       <c r="B8" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
@@ -1019,7 +1087,7 @@
         <v>2</v>
       </c>
       <c r="B9" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
@@ -1027,7 +1095,7 @@
         <v>2</v>
       </c>
       <c r="B10" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
@@ -1035,7 +1103,7 @@
         <v>2</v>
       </c>
       <c r="B11" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
@@ -1043,7 +1111,7 @@
         <v>2</v>
       </c>
       <c r="B12" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
@@ -1051,7 +1119,7 @@
         <v>2</v>
       </c>
       <c r="B13" t="s">
-        <v>14</v>
+        <v>127</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
@@ -1059,7 +1127,7 @@
         <v>2</v>
       </c>
       <c r="B14" t="s">
-        <v>15</v>
+        <v>128</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
@@ -1067,7 +1135,7 @@
         <v>2</v>
       </c>
       <c r="B15" t="s">
-        <v>16</v>
+        <v>129</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
@@ -1075,7 +1143,7 @@
         <v>2</v>
       </c>
       <c r="B16" t="s">
-        <v>17</v>
+        <v>130</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
@@ -1083,7 +1151,7 @@
         <v>2</v>
       </c>
       <c r="B17" t="s">
-        <v>18</v>
+        <v>134</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
@@ -1091,474 +1159,643 @@
         <v>2</v>
       </c>
       <c r="B18" t="s">
-        <v>19</v>
+        <v>135</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="B19" t="s">
-        <v>21</v>
+        <v>131</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="B20" t="s">
-        <v>22</v>
+        <v>132</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="B21" t="s">
-        <v>23</v>
+        <v>133</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="B22" t="s">
-        <v>13</v>
+        <v>136</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="B23" t="s">
-        <v>24</v>
+        <v>137</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="B24" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="B25" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="B26" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="B27" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="B28" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="B29" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="B30" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="B31" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="B32" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="B33" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="B34" t="s">
-        <v>13</v>
+        <v>147</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="B35" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="B36" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B37" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B38" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B39" t="s">
-        <v>16</v>
+        <v>4</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B40" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B41" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B42" t="s">
-        <v>19</v>
+        <v>141</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B43" t="s">
-        <v>13</v>
+        <v>142</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B44" t="s">
-        <v>24</v>
+        <v>143</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B45" t="s">
-        <v>29</v>
+        <v>144</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="B46" t="s">
-        <v>27</v>
+        <v>145</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="B47" t="s">
-        <v>14</v>
+        <v>146</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="B48" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B49" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B50" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B51" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B52" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B53" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B54" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B55" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B56" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B57" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B58" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B59" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B60" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B61" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B62" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B63" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B64" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B65" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B66" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B67" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B68" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B69" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B70" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B71" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B72" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B73" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B74" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B75" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
+        <v>30</v>
+      </c>
+      <c r="B76" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
+        <v>30</v>
+      </c>
+      <c r="B77" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
+        <v>31</v>
+      </c>
+      <c r="B78" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
+        <v>31</v>
+      </c>
+      <c r="B79" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
+        <v>31</v>
+      </c>
+      <c r="B80" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
+        <v>31</v>
+      </c>
+      <c r="B81" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
+        <v>31</v>
+      </c>
+      <c r="B82" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
+        <v>31</v>
+      </c>
+      <c r="B83" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A84" t="s">
+        <v>31</v>
+      </c>
+      <c r="B84" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
+        <v>31</v>
+      </c>
+      <c r="B85" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A86" t="s">
+        <v>31</v>
+      </c>
+      <c r="B86" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A87" t="s">
+        <v>31</v>
+      </c>
+      <c r="B87" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
         <v>32</v>
       </c>
-      <c r="B76" t="s">
+      <c r="B88" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A89" t="s">
+        <v>32</v>
+      </c>
+      <c r="B89" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A90" t="s">
+        <v>32</v>
+      </c>
+      <c r="B90" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A91" t="s">
+        <v>32</v>
+      </c>
+      <c r="B91" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
+        <v>32</v>
+      </c>
+      <c r="B92" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A93" t="s">
+        <v>32</v>
+      </c>
+      <c r="B93" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
+        <v>32</v>
+      </c>
+      <c r="B94" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
+        <v>32</v>
+      </c>
+      <c r="B95" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A96" t="s">
+        <v>32</v>
+      </c>
+      <c r="B96" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A97" t="s">
+        <v>32</v>
+      </c>
+      <c r="B97" t="s">
         <v>27</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:B1" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
debug llamaada a sinónimos en pruebas_explorar_2.ipynb
</commit_message>
<xml_diff>
--- a/data/utilities/stopwords.xlsx
+++ b/data/utilities/stopwords.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP ENVY\Documents\Maestria_MINE\SEMESTRE 4\3.OpcionGrado--Wilmer\capstonenlpencuestas_mine9\data\utilities\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEDDEC1E-A5C8-4DC5-904C-0D37DC84C3F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C64166F5-84E4-4ABE-979E-E8FD0361B271}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="globales" sheetId="2" r:id="rId1"/>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">globales!$A$1:$B$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">particulares!$A$1:$B$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">particulares!$A$1:$B$138</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="157">
   <si>
     <t>encuesta</t>
   </si>
@@ -39,9 +39,6 @@
     <t>palabra</t>
   </si>
   <si>
-    <t>stopwords_evaluaciondocente</t>
-  </si>
-  <si>
     <t>evaluacion</t>
   </si>
   <si>
@@ -93,9 +90,6 @@
     <t>oportunidades de mejora</t>
   </si>
   <si>
-    <t>stopwords_autoevaluaciondocente</t>
-  </si>
-  <si>
     <t>resultados aprendizaje</t>
   </si>
   <si>
@@ -111,27 +105,12 @@
     <t>estudiantes</t>
   </si>
   <si>
-    <t>stopwords_calidaddocentes</t>
-  </si>
-  <si>
     <t>servicio</t>
   </si>
   <si>
-    <t>stopwords_calidadadministrativos</t>
-  </si>
-  <si>
     <t>deberian</t>
   </si>
   <si>
-    <t>stopwords_calidadestudiantes</t>
-  </si>
-  <si>
-    <t>stopwords_calidaddirectivos</t>
-  </si>
-  <si>
-    <t>stopwords_calidadegresados</t>
-  </si>
-  <si>
     <t>stopwords_global</t>
   </si>
   <si>
@@ -478,6 +457,51 @@
   </si>
   <si>
     <t>na</t>
+  </si>
+  <si>
+    <t>estudiante</t>
+  </si>
+  <si>
+    <t>profes</t>
+  </si>
+  <si>
+    <t>emerita</t>
+  </si>
+  <si>
+    <t>emerito</t>
+  </si>
+  <si>
+    <t>enseñante</t>
+  </si>
+  <si>
+    <t>clase</t>
+  </si>
+  <si>
+    <t>curso</t>
+  </si>
+  <si>
+    <t>cursos</t>
+  </si>
+  <si>
+    <t>Evaluación Docente</t>
+  </si>
+  <si>
+    <t>Autoevaluación Docente</t>
+  </si>
+  <si>
+    <t>Calidad Docentes</t>
+  </si>
+  <si>
+    <t>Calidad Administrativos</t>
+  </si>
+  <si>
+    <t>Calidad Estudiantes</t>
+  </si>
+  <si>
+    <t>Calidad Directivos</t>
+  </si>
+  <si>
+    <t>Calidad Egresados</t>
   </si>
 </sst>
 </file>
@@ -812,194 +836,194 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B2" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B4" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B5" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B6" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B7" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B8" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B9" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B10" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B11" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B12" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B13" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B14" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B15" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B17" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B18" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B19" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B20" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B21" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B22" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B23" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B24" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B25" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -1011,10 +1035,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B97"/>
+  <dimension ref="A1:B138"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="30.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.90625" customWidth="1"/>
     <col min="2" max="2" width="24.26953125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1028,774 +1052,1101 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B2" t="s">
         <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="B3" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="B4" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="B5" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="B6" t="s">
-        <v>4</v>
+        <v>144</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="B7" t="s">
-        <v>5</v>
+        <v>145</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="B8" t="s">
-        <v>6</v>
+        <v>146</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="B9" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="B10" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="B11" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="B12" t="s">
-        <v>10</v>
+        <v>143</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="B13" t="s">
-        <v>127</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="B14" t="s">
-        <v>128</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="B15" t="s">
-        <v>129</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="B16" t="s">
-        <v>130</v>
+        <v>9</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="B17" t="s">
-        <v>134</v>
+        <v>120</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="B18" t="s">
-        <v>135</v>
+        <v>121</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="B19" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="B20" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="B21" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="B22" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="B23" t="s">
-        <v>137</v>
+        <v>124</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="B24" t="s">
-        <v>11</v>
+        <v>125</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="B25" t="s">
-        <v>12</v>
+        <v>126</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="B26" t="s">
-        <v>13</v>
+        <v>129</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="B27" t="s">
-        <v>14</v>
+        <v>130</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="B28" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="B29" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="B30" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="B31" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>2</v>
+        <v>150</v>
       </c>
       <c r="B32" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>20</v>
+        <v>150</v>
       </c>
       <c r="B33" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>20</v>
+        <v>150</v>
       </c>
       <c r="B34" t="s">
-        <v>147</v>
+        <v>16</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>20</v>
+        <v>150</v>
       </c>
       <c r="B35" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>20</v>
+        <v>150</v>
       </c>
       <c r="B36" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>20</v>
+        <v>150</v>
       </c>
       <c r="B37" t="s">
-        <v>13</v>
+        <v>134</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>20</v>
+        <v>150</v>
       </c>
       <c r="B38" t="s">
-        <v>24</v>
+        <v>135</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>20</v>
+        <v>150</v>
       </c>
       <c r="B39" t="s">
-        <v>4</v>
+        <v>136</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>20</v>
+        <v>150</v>
       </c>
       <c r="B40" t="s">
-        <v>18</v>
+        <v>137</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>20</v>
+        <v>150</v>
       </c>
       <c r="B41" t="s">
-        <v>19</v>
+        <v>138</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>20</v>
+        <v>150</v>
       </c>
       <c r="B42" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>20</v>
+        <v>150</v>
       </c>
       <c r="B43" t="s">
-        <v>142</v>
+        <v>23</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>20</v>
+        <v>150</v>
       </c>
       <c r="B44" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>20</v>
+        <v>151</v>
       </c>
       <c r="B45" t="s">
-        <v>144</v>
+        <v>19</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>20</v>
+        <v>151</v>
       </c>
       <c r="B46" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
+        <v>151</v>
+      </c>
+      <c r="B47" t="s">
         <v>20</v>
-      </c>
-      <c r="B47" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>20</v>
+        <v>151</v>
       </c>
       <c r="B48" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>26</v>
+        <v>151</v>
       </c>
       <c r="B49" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>26</v>
+        <v>151</v>
       </c>
       <c r="B50" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>26</v>
+        <v>151</v>
       </c>
       <c r="B51" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>26</v>
+        <v>151</v>
       </c>
       <c r="B52" t="s">
-        <v>17</v>
+        <v>131</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>26</v>
+        <v>151</v>
       </c>
       <c r="B53" t="s">
-        <v>18</v>
+        <v>132</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>26</v>
+        <v>151</v>
       </c>
       <c r="B54" t="s">
-        <v>19</v>
+        <v>133</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>26</v>
+        <v>151</v>
       </c>
       <c r="B55" t="s">
-        <v>13</v>
+        <v>144</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>26</v>
+        <v>151</v>
       </c>
       <c r="B56" t="s">
-        <v>24</v>
+        <v>145</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>26</v>
+        <v>151</v>
       </c>
       <c r="B57" t="s">
-        <v>27</v>
+        <v>146</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>28</v>
+        <v>151</v>
       </c>
       <c r="B58" t="s">
-        <v>14</v>
+        <v>3</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>28</v>
+        <v>151</v>
       </c>
       <c r="B59" t="s">
-        <v>15</v>
+        <v>4</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>28</v>
+        <v>151</v>
       </c>
       <c r="B60" t="s">
-        <v>16</v>
+        <v>5</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>28</v>
+        <v>151</v>
       </c>
       <c r="B61" t="s">
-        <v>17</v>
+        <v>143</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>28</v>
+        <v>151</v>
       </c>
       <c r="B62" t="s">
-        <v>18</v>
+        <v>6</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>28</v>
+        <v>151</v>
       </c>
       <c r="B63" t="s">
-        <v>19</v>
+        <v>7</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>28</v>
+        <v>151</v>
       </c>
       <c r="B64" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>28</v>
+        <v>151</v>
       </c>
       <c r="B65" t="s">
-        <v>24</v>
+        <v>9</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>28</v>
+        <v>151</v>
       </c>
       <c r="B66" t="s">
-        <v>29</v>
+        <v>120</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>28</v>
+        <v>151</v>
       </c>
       <c r="B67" t="s">
-        <v>27</v>
+        <v>121</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>30</v>
+        <v>151</v>
       </c>
       <c r="B68" t="s">
-        <v>14</v>
+        <v>122</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>30</v>
+        <v>151</v>
       </c>
       <c r="B69" t="s">
-        <v>15</v>
+        <v>123</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>30</v>
+        <v>151</v>
       </c>
       <c r="B70" t="s">
-        <v>16</v>
+        <v>127</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>30</v>
+        <v>151</v>
       </c>
       <c r="B71" t="s">
-        <v>17</v>
+        <v>128</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>30</v>
+        <v>151</v>
       </c>
       <c r="B72" t="s">
-        <v>18</v>
+        <v>124</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>30</v>
+        <v>151</v>
       </c>
       <c r="B73" t="s">
-        <v>19</v>
+        <v>125</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>30</v>
+        <v>151</v>
       </c>
       <c r="B74" t="s">
-        <v>13</v>
+        <v>126</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>30</v>
+        <v>151</v>
       </c>
       <c r="B75" t="s">
-        <v>24</v>
+        <v>129</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>30</v>
+        <v>151</v>
       </c>
       <c r="B76" t="s">
-        <v>29</v>
+        <v>130</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>30</v>
+        <v>151</v>
       </c>
       <c r="B77" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>31</v>
+        <v>151</v>
       </c>
       <c r="B78" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>31</v>
+        <v>151</v>
       </c>
       <c r="B79" t="s">
-        <v>15</v>
+        <v>134</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>31</v>
+        <v>151</v>
       </c>
       <c r="B80" t="s">
-        <v>16</v>
+        <v>135</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
-        <v>31</v>
+        <v>151</v>
       </c>
       <c r="B81" t="s">
-        <v>17</v>
+        <v>136</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>31</v>
+        <v>151</v>
       </c>
       <c r="B82" t="s">
-        <v>18</v>
+        <v>137</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
-        <v>31</v>
+        <v>151</v>
       </c>
       <c r="B83" t="s">
-        <v>19</v>
+        <v>138</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
-        <v>31</v>
+        <v>151</v>
       </c>
       <c r="B84" t="s">
-        <v>13</v>
+        <v>139</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
-        <v>31</v>
+        <v>151</v>
       </c>
       <c r="B85" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
-        <v>31</v>
+        <v>151</v>
       </c>
       <c r="B86" t="s">
-        <v>29</v>
+        <v>142</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
-        <v>31</v>
+        <v>151</v>
       </c>
       <c r="B87" t="s">
-        <v>27</v>
+        <v>147</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
-        <v>32</v>
+        <v>151</v>
       </c>
       <c r="B88" t="s">
-        <v>14</v>
+        <v>148</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
-        <v>32</v>
+        <v>151</v>
       </c>
       <c r="B89" t="s">
-        <v>15</v>
+        <v>149</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
-        <v>32</v>
+        <v>152</v>
       </c>
       <c r="B90" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
-        <v>32</v>
+        <v>152</v>
       </c>
       <c r="B91" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
-        <v>32</v>
+        <v>152</v>
       </c>
       <c r="B92" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
-        <v>32</v>
+        <v>152</v>
       </c>
       <c r="B93" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
-        <v>32</v>
+        <v>152</v>
       </c>
       <c r="B94" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
-        <v>32</v>
+        <v>152</v>
       </c>
       <c r="B95" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
-        <v>32</v>
+        <v>152</v>
       </c>
       <c r="B96" t="s">
-        <v>29</v>
+        <v>12</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
-        <v>32</v>
+        <v>152</v>
       </c>
       <c r="B97" t="s">
-        <v>27</v>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A98" t="s">
+        <v>152</v>
+      </c>
+      <c r="B98" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A99" t="s">
+        <v>153</v>
+      </c>
+      <c r="B99" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A100" t="s">
+        <v>153</v>
+      </c>
+      <c r="B100" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A101" t="s">
+        <v>153</v>
+      </c>
+      <c r="B101" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A102" t="s">
+        <v>153</v>
+      </c>
+      <c r="B102" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A103" t="s">
+        <v>153</v>
+      </c>
+      <c r="B103" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A104" t="s">
+        <v>153</v>
+      </c>
+      <c r="B104" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A105" t="s">
+        <v>153</v>
+      </c>
+      <c r="B105" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A106" t="s">
+        <v>153</v>
+      </c>
+      <c r="B106" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A107" t="s">
+        <v>153</v>
+      </c>
+      <c r="B107" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A108" t="s">
+        <v>153</v>
+      </c>
+      <c r="B108" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A109" t="s">
+        <v>154</v>
+      </c>
+      <c r="B109" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A110" t="s">
+        <v>154</v>
+      </c>
+      <c r="B110" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A111" t="s">
+        <v>154</v>
+      </c>
+      <c r="B111" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A112" t="s">
+        <v>154</v>
+      </c>
+      <c r="B112" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A113" t="s">
+        <v>154</v>
+      </c>
+      <c r="B113" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A114" t="s">
+        <v>154</v>
+      </c>
+      <c r="B114" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A115" t="s">
+        <v>154</v>
+      </c>
+      <c r="B115" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A116" t="s">
+        <v>154</v>
+      </c>
+      <c r="B116" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A117" t="s">
+        <v>154</v>
+      </c>
+      <c r="B117" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A118" t="s">
+        <v>154</v>
+      </c>
+      <c r="B118" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A119" t="s">
+        <v>155</v>
+      </c>
+      <c r="B119" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A120" t="s">
+        <v>155</v>
+      </c>
+      <c r="B120" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A121" t="s">
+        <v>155</v>
+      </c>
+      <c r="B121" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A122" t="s">
+        <v>155</v>
+      </c>
+      <c r="B122" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A123" t="s">
+        <v>155</v>
+      </c>
+      <c r="B123" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A124" t="s">
+        <v>155</v>
+      </c>
+      <c r="B124" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A125" t="s">
+        <v>155</v>
+      </c>
+      <c r="B125" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A126" t="s">
+        <v>155</v>
+      </c>
+      <c r="B126" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A127" t="s">
+        <v>155</v>
+      </c>
+      <c r="B127" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A128" t="s">
+        <v>155</v>
+      </c>
+      <c r="B128" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A129" t="s">
+        <v>156</v>
+      </c>
+      <c r="B129" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A130" t="s">
+        <v>156</v>
+      </c>
+      <c r="B130" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A131" t="s">
+        <v>156</v>
+      </c>
+      <c r="B131" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A132" t="s">
+        <v>156</v>
+      </c>
+      <c r="B132" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A133" t="s">
+        <v>156</v>
+      </c>
+      <c r="B133" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A134" t="s">
+        <v>156</v>
+      </c>
+      <c r="B134" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A135" t="s">
+        <v>156</v>
+      </c>
+      <c r="B135" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A136" t="s">
+        <v>156</v>
+      </c>
+      <c r="B136" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A137" t="s">
+        <v>156</v>
+      </c>
+      <c r="B137" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A138" t="s">
+        <v>156</v>
+      </c>
+      <c r="B138" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B1" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1815,562 +2166,562 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B2" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B3" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B4" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B5" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B6" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B7" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B8" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" t="s">
         <v>61</v>
-      </c>
-      <c r="B9" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B10" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B11" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B12" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B13" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B14" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B15" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B16" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B17" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B18" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B19" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B20" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B21" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B22" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B23" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B24" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B25" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B26" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B27" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B28" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B29" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B30" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B31" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B32" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B33" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B34" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B35" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B36" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B37" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B38" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B39" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B40" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B41" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B42" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B43" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B44" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B45" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B46" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B47" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B48" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B49" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B50" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B51" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B52" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B53" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B54" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B55" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B56" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B57" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B58" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B59" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B60" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B61" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B62" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B63" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B64" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B65" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B66" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B67" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B68" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B69" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B70" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="B71" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>